<commit_message>
Implement UI test uniqueness enforcement with duplicate detection - Added script normalization and URL case handling
</commit_message>
<xml_diff>
--- a/data/api_tests.xlsx
+++ b/data/api_tests.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N6"/>
+  <dimension ref="A1:N14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -581,7 +581,6 @@
           <t>http://localhost:8012/users/me</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>{"Content-Type": "application/json", "Authorization": "Bearer "}</t>
@@ -649,8 +648,6 @@
           <t>http://localhost:8012/products?limit=10</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>200</t>
@@ -743,7 +740,6 @@
           <t>*</t>
         </is>
       </c>
-      <c r="K5" t="inlineStr"/>
       <c r="L5" t="inlineStr">
         <is>
           <t>active</t>
@@ -781,8 +777,6 @@
           <t>http://localhost:8012/health</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
         <is>
           <t>200</t>
@@ -823,6 +817,456 @@
           <t>PASS</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (number)</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>{"name": 123, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (boolean)</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>{"name": true, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (number)</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/create</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>{"name": 123, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (boolean)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/new</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>{"name": true, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (number)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/validate/number</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>{"name": 123, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Create user - invalid name type (boolean)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/validate/boolean</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>{"name": true, "email": "test@example.com"}</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Create user - empty body not allowed</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/validate/empty</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Users</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Create user - empty body not allowed</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>POST</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>http://localhost:8012/users/validate/empty</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>{"Content-Type": "application/json"}</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>400</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>detail</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>*</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2025-11-07 23:19</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>